<commit_message>
fix: balancete Formosa — SaldoAnterior, flags S/N, Conta Aux., atualiza MOLDES
Problema 1 — SaldoAnterior NaN para todas as contas:
  substitui fallback sa_col+1 por scan range (sa_col … debito-1), tornando
  a leitura robusta para qualquer variação do offset TOTVS.

Problema 2 — Flags Estoque/ContaFinanceira/ReservaDeContingência sempre 'N':
  quando a planilha-fonte não tem colunas de flag, aplica regras baseadas
  em prefixo de conta conforme plano de contas IMED:
    Estoque='S' para 1.1.5.x
    ContaFinanceira='S' para 1.1.1.02.02.x e 1.1.1.02.04.x
    ReservaDeContingência='S' para 1.1.1.02.02.012 e 1.1.1.02.04.010

Problema 3 — 550 linhas "Conta Aux.:" indevidas no output:
  adiciona filtro `conta_norm.startswith("conta aux")` em parse_balancete_rows.

Atualiza MOLDES/BALANCETE.FORMATO.xlsx com as 28 células de flags que
estavam como 'N' mas devem ser 'S' conforme as regras recém-definidas.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MOLDES/BALANCETE.FORMATO.xlsx
+++ b/MOLDES/BALANCETE.FORMATO.xlsx
@@ -853,7 +853,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="M8" s="2" t="n"/>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -2854,7 +2854,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: balancete — backward SA scan, ReservaDeContingência por keyword
SaldoAnterior: substitui forward scan (sa_col→deb_col) por backward scan
(deb_col-1→desc_col), eliminando paradas prematuras em coluna filler zero.

ReservaDeContingência: quando não há coluna na fonte, detecta por keyword
('fundo', 'reserva', 'contingencia') no NomeConta, para contas sob
1.1.1.02.02.x e 1.1.1.02.04.x — funciona em todas as unidades sem lista
hardcoded. MOLDES FORMATO atualizado: 2 contas FUNDO agora = 'S'.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MOLDES/BALANCETE.FORMATO.xlsx
+++ b/MOLDES/BALANCETE.FORMATO.xlsx
@@ -984,7 +984,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="M8" s="2" t="n"/>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>

</xml_diff>